<commit_message>
fix(nlp): skip compliment-only phrases in bad-review keywords
Also sync pipeline, docs, weather export, and refresh tracked raw exports
(remove superseded xlsx snapshots; update 菜品库 snapshot).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/夕佳悦/夕佳悦餐厅_园博馆店_菜品库_20260427_1022_a645046d_1777256566986.xlsx
+++ b/data/夕佳悦/夕佳悦餐厅_园博馆店_菜品库_20260427_1022_a645046d_1777256566986.xlsx
@@ -1,57 +1,103 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/weixin/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{819CF77B-9AC0-6243-9A31-71DDE8C4D884}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="29100" windowHeight="12160"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="198">
+  <si>
+    <t>序号</t>
+  </si>
   <si>
     <t>菜品名称</t>
   </si>
   <si>
+    <t>菜品分类</t>
+  </si>
+  <si>
+    <t>菜品类型</t>
+  </si>
+  <si>
+    <t>价格</t>
+  </si>
+  <si>
+    <t>菜品状态</t>
+  </si>
+  <si>
     <t>红烩牛腩焗意面（2-3人份）</t>
   </si>
   <si>
     <t>主餐（意面、焗饭）</t>
   </si>
   <si>
+    <t>普通菜</t>
+  </si>
+  <si>
+    <t>￥98.00</t>
+  </si>
+  <si>
+    <t>在售</t>
+  </si>
+  <si>
     <t>浓汤番茄焗意面（2-3人份）</t>
   </si>
   <si>
+    <t>￥88.00</t>
+  </si>
+  <si>
     <t>意式肉酱焗意面（2-3人份）</t>
   </si>
   <si>
     <t>奶油蘑菇意面</t>
   </si>
   <si>
+    <t>￥42.00</t>
+  </si>
+  <si>
     <t>传统意式肉酱面</t>
   </si>
   <si>
+    <t>￥38.00</t>
+  </si>
+  <si>
     <t>传统番茄海鲜意面（微辣）</t>
   </si>
   <si>
+    <t>￥48.00</t>
+  </si>
+  <si>
     <t>海鲜炒乌冬面</t>
   </si>
   <si>
     <t>新儿童餐肉酱面</t>
   </si>
   <si>
+    <t>￥0.00</t>
+  </si>
+  <si>
     <t>新儿童餐红烩泥肠</t>
   </si>
   <si>
@@ -70,9 +116,15 @@
     <t>主菜（肉类）</t>
   </si>
   <si>
+    <t>￥438.00</t>
+  </si>
+  <si>
     <t>美式烟熏猪肋排</t>
   </si>
   <si>
+    <t>￥198.00</t>
+  </si>
+  <si>
     <t>脆皮烤春鸡</t>
   </si>
   <si>
@@ -82,6 +134,9 @@
     <t>香烤薄饼</t>
   </si>
   <si>
+    <t>￥46.00</t>
+  </si>
+  <si>
     <t>金枪鱼薄饼</t>
   </si>
   <si>
@@ -112,6 +167,9 @@
     <t>甜品</t>
   </si>
   <si>
+    <t>￥32.00</t>
+  </si>
+  <si>
     <t>伯爵焦糖巴斯克</t>
   </si>
   <si>
@@ -124,6 +182,9 @@
     <t>天福料多多（特色饮料）</t>
   </si>
   <si>
+    <t>￥28.00</t>
+  </si>
+  <si>
     <t>巧克力</t>
   </si>
   <si>
@@ -145,6 +206,9 @@
     <t>沙拉</t>
   </si>
   <si>
+    <t>￥58.00</t>
+  </si>
+  <si>
     <t>金枪鱼沙拉</t>
   </si>
   <si>
@@ -154,6 +218,9 @@
     <t>开胃菜（小食、炸物）</t>
   </si>
   <si>
+    <t>￥108.00</t>
+  </si>
+  <si>
     <t>天福烤翅（3对）</t>
   </si>
   <si>
@@ -163,6 +230,9 @@
     <t>缤纷小食总汇</t>
   </si>
   <si>
+    <t>￥78.00</t>
+  </si>
+  <si>
     <t>芝香火腿焗豆泥</t>
   </si>
   <si>
@@ -175,6 +245,9 @@
     <t>经典咖啡</t>
   </si>
   <si>
+    <t>￥35.00</t>
+  </si>
+  <si>
     <t>拿铁</t>
   </si>
   <si>
@@ -208,6 +281,9 @@
     <t>大师咖啡</t>
   </si>
   <si>
+    <t>￥39.00</t>
+  </si>
+  <si>
     <t>天福甄烤酱肘子焗饭</t>
   </si>
   <si>
@@ -235,6 +311,9 @@
     <t>中国茶（壶）赠送时令茶食</t>
   </si>
   <si>
+    <t>￥68.00</t>
+  </si>
+  <si>
     <t>茉莉花茶-银针（壶）</t>
   </si>
   <si>
@@ -259,21 +338,33 @@
     <t>吮指鱼块</t>
   </si>
   <si>
+    <t>￥36.00</t>
+  </si>
+  <si>
     <t>厚烤安格斯肉眼牛排</t>
   </si>
   <si>
+    <t>￥188.00</t>
+  </si>
+  <si>
     <t>蒲烧鳗鱼饭</t>
   </si>
   <si>
     <t>蒜香面包</t>
   </si>
   <si>
+    <t>￥18.00</t>
+  </si>
+  <si>
     <t>天福甄烤酱肘子薄饼</t>
   </si>
   <si>
     <t>美团团购套餐</t>
   </si>
   <si>
+    <t>￥52.00</t>
+  </si>
+  <si>
     <t>天福小香肠薄饼</t>
   </si>
   <si>
@@ -298,9 +389,15 @@
     <t>美团团购-【茶香四溢】中国茶4选1+黑松露薯条套餐</t>
   </si>
   <si>
+    <t>套餐</t>
+  </si>
+  <si>
     <t>美团团购-【品味西韵】美式咖啡+蒜香面包单人餐</t>
   </si>
   <si>
+    <t>￥29.80</t>
+  </si>
+  <si>
     <t>咖喱鸡肉饭</t>
   </si>
   <si>
@@ -328,6 +425,9 @@
     <t>厚烤安格斯肉眼牛排（单人份）</t>
   </si>
   <si>
+    <t>￥180.00</t>
+  </si>
+  <si>
     <t>美团团购-【甄选主食】西餐单人餐｜酱肘子/小香肠/咖喱鸡（含饮品）-251107121910</t>
   </si>
   <si>
@@ -364,12 +464,21 @@
     <t>美团团购-【悦享】经典双人餐</t>
   </si>
   <si>
+    <t>￥228.00</t>
+  </si>
+  <si>
     <t>美团团购-【悦惠】管饱双人餐</t>
   </si>
   <si>
+    <t>￥268.00</t>
+  </si>
+  <si>
     <t>美团团购-【饕餮肉食】欢聚4人餐｜甄选肉食混拼+缤纷小食总汇</t>
   </si>
   <si>
+    <t>￥568.00</t>
+  </si>
+  <si>
     <t>黑芝麻巴斯克</t>
   </si>
   <si>
@@ -379,6 +488,9 @@
     <t>米饭</t>
   </si>
   <si>
+    <t>￥3.00</t>
+  </si>
+  <si>
     <t>美团团购-【悦惠】管饱双人餐-251214102133</t>
   </si>
   <si>
@@ -421,12 +533,21 @@
     <t>饮料</t>
   </si>
   <si>
+    <t>￥15.00</t>
+  </si>
+  <si>
     <t>含汽姜汁柠檬汁（瓶）</t>
   </si>
   <si>
+    <t>￥12.00</t>
+  </si>
+  <si>
     <t>捏爆甜橙汁（冷）</t>
   </si>
   <si>
+    <t>￥20.00</t>
+  </si>
+  <si>
     <t>捏爆苹果汁（冷）</t>
   </si>
   <si>
@@ -496,149 +617,378 @@
     <t>赵州雪梨汁（瓶）</t>
   </si>
   <si>
-    <t>序号</t>
-  </si>
-  <si>
-    <t>菜品分类</t>
-  </si>
-  <si>
-    <t>菜品类型</t>
-  </si>
-  <si>
-    <t>价格</t>
-  </si>
-  <si>
-    <t>菜品状态</t>
-  </si>
-  <si>
-    <t>普通菜</t>
-  </si>
-  <si>
-    <t>￥98.00</t>
-  </si>
-  <si>
-    <t>在售</t>
-  </si>
-  <si>
-    <t>￥88.00</t>
-  </si>
-  <si>
-    <t>￥42.00</t>
-  </si>
-  <si>
-    <t>￥38.00</t>
-  </si>
-  <si>
-    <t>￥48.00</t>
-  </si>
-  <si>
-    <t>￥0.00</t>
-  </si>
-  <si>
-    <t>￥438.00</t>
-  </si>
-  <si>
-    <t>￥198.00</t>
-  </si>
-  <si>
-    <t>￥46.00</t>
-  </si>
-  <si>
-    <t>￥32.00</t>
-  </si>
-  <si>
-    <t>￥28.00</t>
-  </si>
-  <si>
-    <t>￥58.00</t>
-  </si>
-  <si>
-    <t>￥108.00</t>
-  </si>
-  <si>
-    <t>￥78.00</t>
-  </si>
-  <si>
-    <t>￥35.00</t>
-  </si>
-  <si>
-    <t>￥39.00</t>
-  </si>
-  <si>
-    <t>￥68.00</t>
-  </si>
-  <si>
-    <t>￥36.00</t>
-  </si>
-  <si>
-    <t>￥188.00</t>
-  </si>
-  <si>
-    <t>￥18.00</t>
-  </si>
-  <si>
-    <t>￥52.00</t>
-  </si>
-  <si>
-    <t>套餐</t>
-  </si>
-  <si>
-    <t>￥29.80</t>
-  </si>
-  <si>
-    <t>￥180.00</t>
-  </si>
-  <si>
-    <t>￥228.00</t>
-  </si>
-  <si>
-    <t>￥268.00</t>
-  </si>
-  <si>
-    <t>￥568.00</t>
-  </si>
-  <si>
-    <t>￥3.00</t>
-  </si>
-  <si>
-    <t>￥15.00</t>
-  </si>
-  <si>
-    <t>￥12.00</t>
-  </si>
-  <si>
-    <t>￥20.00</t>
+    <t>青柠可尔必思</t>
+  </si>
+  <si>
+    <t>红柚可尔必思</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="8" formatCode="&quot;￥&quot;#,##0.00;[Red]&quot;￥&quot;\-#,##0.00"/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="等线"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="等线"/>
-      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -646,28 +996,317 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -716,7 +1355,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -749,26 +1388,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -801,23 +1423,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -959,38 +1564,36 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CF9693B-2A6E-2E4B-9FB6-7069C59E3F2F}">
-  <dimension ref="A1:F137"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F139"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16.8" outlineLevelCol="5"/>
+  <cols>
+    <col min="2" max="2" width="15.1785714285714" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>158</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>159</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>160</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>161</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>162</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -998,19 +1601,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>164</v>
+        <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1018,19 +1621,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1038,19 +1641,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1058,19 +1661,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1078,19 +1681,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1098,19 +1701,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
         <v>7</v>
       </c>
-      <c r="C7" t="s">
-        <v>2</v>
-      </c>
       <c r="D7" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1118,19 +1721,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1138,19 +1741,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1158,19 +1761,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F10" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1178,19 +1781,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1198,19 +1801,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F12" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1218,19 +1821,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1238,19 +1841,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E14" t="s">
-        <v>171</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1258,19 +1861,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E15" t="s">
-        <v>172</v>
+        <v>31</v>
       </c>
       <c r="F15" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1278,19 +1881,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D16" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E16" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F16" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1298,19 +1901,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E17" t="s">
-        <v>173</v>
+        <v>35</v>
       </c>
       <c r="F17" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1318,19 +1921,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>173</v>
+        <v>35</v>
       </c>
       <c r="F18" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1338,19 +1941,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>173</v>
+        <v>35</v>
       </c>
       <c r="F19" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1358,19 +1961,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E20" t="s">
-        <v>173</v>
+        <v>35</v>
       </c>
       <c r="F20" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1378,19 +1981,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D21" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E21" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F21" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1398,19 +2001,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D22" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E22" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F22" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1418,19 +2021,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="C23" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F23" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1438,19 +2041,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C24" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F24" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1458,19 +2061,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="C25" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D25" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F25" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1478,19 +2081,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D26" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E26" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F26" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1498,19 +2101,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D27" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E27" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F27" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1518,19 +2121,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E28" t="s">
-        <v>175</v>
+        <v>51</v>
       </c>
       <c r="F28" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1538,19 +2141,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="D29" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F29" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1558,19 +2161,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="C30" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="D30" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E30" t="s">
-        <v>175</v>
+        <v>51</v>
       </c>
       <c r="F30" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1578,19 +2181,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="C31" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E31" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1598,19 +2201,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="C32" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D32" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E32" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F32" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1618,19 +2221,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="C33" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="D33" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E33" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F33" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1638,19 +2241,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="C34" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="D34" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E34" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F34" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1658,19 +2261,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C35" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D35" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E35" t="s">
-        <v>177</v>
+        <v>63</v>
       </c>
       <c r="F35" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1678,19 +2281,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="C36" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D36" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E36" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1698,19 +2301,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C37" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D37" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E37" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F37" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1718,19 +2321,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C38" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D38" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E38" t="s">
-        <v>178</v>
+        <v>67</v>
       </c>
       <c r="F38" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1738,19 +2341,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="C39" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D39" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E39" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F39" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1758,19 +2361,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D40" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E40" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F40" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1778,19 +2381,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="C41" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="D41" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E41" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="F41" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1798,19 +2401,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="C42" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="D42" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E42" t="s">
-        <v>179</v>
+        <v>72</v>
       </c>
       <c r="F42" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1818,19 +2421,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C43" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="D43" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E43" t="s">
-        <v>175</v>
+        <v>51</v>
       </c>
       <c r="F43" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1838,19 +2441,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C44" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="D44" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E44" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F44" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -1858,19 +2461,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="C45" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F45" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1878,19 +2481,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="C46" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D46" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E46" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F46" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -1898,19 +2501,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="C47" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D47" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E47" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F47" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1918,19 +2521,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="C48" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="D48" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E48" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F48" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1938,19 +2541,19 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="C49" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="D49" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E49" t="s">
-        <v>180</v>
+        <v>84</v>
       </c>
       <c r="F49" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -1958,19 +2561,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C50" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D50" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E50" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F50" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -1978,19 +2581,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C51" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D51" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E51" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F51" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -1998,19 +2601,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="C52" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="D52" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E52" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F52" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2018,19 +2621,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C53" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D53" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E53" t="s">
-        <v>175</v>
+        <v>51</v>
       </c>
       <c r="F53" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2038,19 +2641,19 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C54" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D54" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E54" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F54" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2058,19 +2661,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D55" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E55" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F55" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2078,19 +2681,19 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="C56" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="D56" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E56" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F56" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2098,19 +2701,19 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="C57" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="D57" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E57" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F57" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2118,19 +2721,19 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="C58" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="D58" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E58" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F58" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2138,19 +2741,19 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="C59" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="D59" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E59" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F59" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2158,19 +2761,19 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E60" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F60" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2178,19 +2781,19 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="C61" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="D61" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E61" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F61" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -2198,19 +2801,19 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="C62" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D62" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E62" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F62" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -2218,19 +2821,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="C63" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D63" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E63" t="s">
-        <v>182</v>
+        <v>103</v>
       </c>
       <c r="F63" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2238,19 +2841,19 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="C64" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D64" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E64" t="s">
-        <v>183</v>
+        <v>105</v>
       </c>
       <c r="F64" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2258,19 +2861,19 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="C65" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D65" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E65" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F65" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2278,19 +2881,19 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="C66" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D66" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E66" t="s">
-        <v>184</v>
+        <v>108</v>
       </c>
       <c r="F66" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2298,19 +2901,19 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="C67" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D67" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E67" t="s">
-        <v>185</v>
+        <v>111</v>
       </c>
       <c r="F67" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2318,19 +2921,19 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>84</v>
+        <v>112</v>
       </c>
       <c r="C68" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D68" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E68" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F68" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -2338,19 +2941,19 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="C69" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D69" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E69" t="s">
-        <v>175</v>
+        <v>51</v>
       </c>
       <c r="F69" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -2358,19 +2961,19 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="C70" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D70" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E70" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F70" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -2378,19 +2981,19 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="C71" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D71" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E71" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F71" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -2398,19 +3001,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="C72" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D72" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E72" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F72" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -2418,19 +3021,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="C73" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D73" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E73" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F73" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -2438,19 +3041,19 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="C74" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D74" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E74" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F74" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -2458,19 +3061,19 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>91</v>
+        <v>119</v>
       </c>
       <c r="C75" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D75" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E75" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F75" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -2478,19 +3081,19 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="C76" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D76" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E76" t="s">
-        <v>187</v>
+        <v>122</v>
       </c>
       <c r="F76" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -2498,19 +3101,19 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="C77" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D77" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E77" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F77" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -2518,19 +3121,19 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="C78" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D78" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E78" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F78" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -2538,19 +3141,19 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="C79" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D79" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E79" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F79" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -2558,19 +3161,19 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="C80" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D80" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E80" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F80" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2578,19 +3181,19 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="C81" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D81" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E81" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F81" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2598,19 +3201,19 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="C82" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D82" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E82" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F82" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2618,19 +3221,19 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="C83" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D83" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E83" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F83" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2638,19 +3241,19 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C84" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D84" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E84" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F84" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -2658,19 +3261,19 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="C85" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D85" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E85" t="s">
-        <v>188</v>
+        <v>132</v>
       </c>
       <c r="F85" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -2678,19 +3281,19 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
       <c r="C86" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D86" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E86" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F86" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -2698,19 +3301,19 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="C87" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D87" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E87" t="s">
-        <v>178</v>
+        <v>67</v>
       </c>
       <c r="F87" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -2718,19 +3321,19 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="C88" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="D88" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E88" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F88" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -2738,19 +3341,19 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="C89" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="D89" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E89" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F89" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -2758,19 +3361,19 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
       <c r="C90" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="D90" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E90" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F90" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -2778,19 +3381,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>108</v>
+        <v>139</v>
       </c>
       <c r="C91" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="D91" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E91" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F91" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -2798,19 +3401,19 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>109</v>
+        <v>140</v>
       </c>
       <c r="C92" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D92" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E92" t="s">
-        <v>178</v>
+        <v>67</v>
       </c>
       <c r="F92" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -2818,19 +3421,19 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>110</v>
+        <v>141</v>
       </c>
       <c r="C93" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D93" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F93" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -2838,19 +3441,19 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>111</v>
+        <v>142</v>
       </c>
       <c r="C94" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D94" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E94" t="s">
-        <v>178</v>
+        <v>67</v>
       </c>
       <c r="F94" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -2858,19 +3461,19 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="C95" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D95" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E95" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F95" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -2878,19 +3481,19 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>113</v>
+        <v>144</v>
       </c>
       <c r="C96" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D96" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E96" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="F96" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -2898,19 +3501,19 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>114</v>
+        <v>146</v>
       </c>
       <c r="C97" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D97" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E97" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F97" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -2918,19 +3521,19 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>115</v>
+        <v>148</v>
       </c>
       <c r="C98" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D98" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E98" t="s">
-        <v>191</v>
+        <v>149</v>
       </c>
       <c r="F98" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -2938,19 +3541,19 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>116</v>
+        <v>150</v>
       </c>
       <c r="C99" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D99" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E99" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="F99" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -2958,19 +3561,19 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="C100" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D100" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E100" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F100" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -2978,19 +3581,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="C101" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D101" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E101" t="s">
-        <v>192</v>
+        <v>153</v>
       </c>
       <c r="F101" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -2998,19 +3601,19 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="C102" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D102" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E102" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F102" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3018,19 +3621,19 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="C103" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D103" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E103" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F103" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3038,19 +3641,19 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="C104" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D104" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E104" t="s">
-        <v>166</v>
+        <v>12</v>
       </c>
       <c r="F104" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3058,19 +3661,19 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="C105" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D105" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E105" t="s">
-        <v>185</v>
+        <v>111</v>
       </c>
       <c r="F105" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3078,19 +3681,19 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="C106" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="D106" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E106" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F106" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3098,19 +3701,19 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="C107" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="D107" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E107" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F107" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3118,19 +3721,19 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="C108" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D108" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E108" t="s">
-        <v>167</v>
+        <v>15</v>
       </c>
       <c r="F108" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3138,19 +3741,19 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="C109" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D109" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E109" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F109" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -3158,19 +3761,19 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
       <c r="C110" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D110" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E110" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="F110" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -3178,19 +3781,19 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
       <c r="C111" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D111" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E111" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F111" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3198,19 +3801,19 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="C112" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D112" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E112" t="s">
-        <v>191</v>
+        <v>149</v>
       </c>
       <c r="F112" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -3218,19 +3821,19 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>131</v>
+        <v>166</v>
       </c>
       <c r="C113" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="D113" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E113" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="F113" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -3238,19 +3841,19 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>133</v>
+        <v>169</v>
       </c>
       <c r="C114" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="D114" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E114" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="F114" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -3258,19 +3861,19 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>134</v>
+        <v>171</v>
       </c>
       <c r="C115" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D115" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E115" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="F115" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -3278,19 +3881,19 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="C116" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D116" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E116" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="F116" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -3298,19 +3901,19 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>136</v>
+        <v>174</v>
       </c>
       <c r="C117" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D117" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E117" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="F117" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -3318,19 +3921,19 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>137</v>
+        <v>175</v>
       </c>
       <c r="C118" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D118" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E118" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="F118" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -3338,19 +3941,19 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>138</v>
+        <v>176</v>
       </c>
       <c r="C119" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D119" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E119" t="s">
-        <v>195</v>
+        <v>172</v>
       </c>
       <c r="F119" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -3358,19 +3961,19 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>139</v>
+        <v>177</v>
       </c>
       <c r="C120" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D120" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E120" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F120" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -3378,19 +3981,19 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>140</v>
+        <v>178</v>
       </c>
       <c r="C121" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D121" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E121" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="F121" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -3398,19 +4001,19 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>141</v>
+        <v>179</v>
       </c>
       <c r="C122" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D122" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E122" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F122" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -3418,19 +4021,19 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="C123" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D123" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E123" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F123" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -3438,19 +4041,19 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="C124" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D124" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E124" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="F124" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -3458,19 +4061,19 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="C125" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D125" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E125" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F125" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -3478,19 +4081,19 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
       <c r="C126" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D126" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E126" t="s">
-        <v>176</v>
+        <v>59</v>
       </c>
       <c r="F126" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -3498,19 +4101,19 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="C127" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D127" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E127" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="F127" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -3518,19 +4121,19 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
+        <v>185</v>
+      </c>
+      <c r="C128" t="s">
+        <v>110</v>
+      </c>
+      <c r="D128" t="s">
+        <v>120</v>
+      </c>
+      <c r="E128" t="s">
         <v>147</v>
       </c>
-      <c r="C128" t="s">
-        <v>83</v>
-      </c>
-      <c r="D128" t="s">
-        <v>186</v>
-      </c>
-      <c r="E128" t="s">
-        <v>190</v>
-      </c>
       <c r="F128" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -3538,19 +4141,19 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>148</v>
+        <v>186</v>
       </c>
       <c r="C129" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D129" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E129" t="s">
-        <v>190</v>
+        <v>147</v>
       </c>
       <c r="F129" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -3558,19 +4161,19 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>149</v>
+        <v>187</v>
       </c>
       <c r="C130" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="D130" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E130" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="F130" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -3578,19 +4181,19 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>151</v>
+        <v>189</v>
       </c>
       <c r="C131" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D131" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E131" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F131" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -3598,19 +4201,19 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
       <c r="C132" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D132" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E132" t="s">
-        <v>170</v>
+        <v>22</v>
       </c>
       <c r="F132" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -3618,19 +4221,19 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>153</v>
+        <v>191</v>
       </c>
       <c r="C133" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="D133" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E133" t="s">
-        <v>181</v>
+        <v>94</v>
       </c>
       <c r="F133" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -3638,19 +4241,19 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>154</v>
+        <v>192</v>
       </c>
       <c r="C134" t="s">
-        <v>150</v>
+        <v>188</v>
       </c>
       <c r="D134" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="E134" t="s">
-        <v>169</v>
+        <v>19</v>
       </c>
       <c r="F134" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -3658,19 +4261,19 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>155</v>
+        <v>193</v>
       </c>
       <c r="C135" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="D135" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E135" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="F135" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -3678,19 +4281,19 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>156</v>
+        <v>194</v>
       </c>
       <c r="C136" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="D136" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E136" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="F136" t="s">
-        <v>165</v>
+        <v>10</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -3698,23 +4301,63 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="C137" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="D137" t="s">
-        <v>163</v>
+        <v>8</v>
       </c>
       <c r="E137" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="F137" t="s">
-        <v>165</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>196</v>
+      </c>
+      <c r="C138" t="s">
+        <v>89</v>
+      </c>
+      <c r="D138" t="s">
+        <v>8</v>
+      </c>
+      <c r="E138" s="1">
+        <v>28</v>
+      </c>
+      <c r="F138" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>197</v>
+      </c>
+      <c r="C139" t="s">
+        <v>89</v>
+      </c>
+      <c r="D139" t="s">
+        <v>8</v>
+      </c>
+      <c r="E139" s="1">
+        <v>28</v>
+      </c>
+      <c r="F139" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
weekly update: 追加 2026-07-27 周两店经营看板数据
同步最新源表与天气，营收/订单对账通过后更新线上看板。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/夕佳悦/夕佳悦餐厅_园博馆店_菜品库_20260427_1022_a645046d_1777256566986.xlsx
+++ b/data/夕佳悦/夕佳悦餐厅_园博馆店_菜品库_20260427_1022_a645046d_1777256566986.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="233">
   <si>
     <t>序号</t>
   </si>
@@ -494,24 +494,12 @@
     <t>生椰汁（冷）</t>
   </si>
   <si>
-    <t>玫瑰汤圆美式</t>
-  </si>
-  <si>
-    <t>红楼赏味</t>
-  </si>
-  <si>
     <t>牡丹花糕</t>
   </si>
   <si>
     <t>五红粥</t>
   </si>
   <si>
-    <t>红楼赏味下午茶</t>
-  </si>
-  <si>
-    <t>红楼赏味养生粥+主食薄饼</t>
-  </si>
-  <si>
     <t>西柚味苏打水（瓶）</t>
   </si>
   <si>
@@ -729,6 +717,15 @@
   </si>
   <si>
     <t>儿童餐蝴蝶面</t>
+  </si>
+  <si>
+    <t>美式咖啡（热）</t>
+  </si>
+  <si>
+    <t>美式咖啡（冰）</t>
+  </si>
+  <si>
+    <t>美团团购-【品味西韵】美式咖啡+蒜香面包单人餐-260802170254</t>
   </si>
 </sst>
 </file>
@@ -750,10 +747,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FF222222"/>
-      <name val="Helvetica Neue"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1691,7 +1689,7 @@
     <col min="5" max="5" width="11.0666666666667"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.4" spans="1:6">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1711,7 +1709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="20.4" spans="1:6">
+    <row r="2" spans="1:6">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1731,7 +1729,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="20.4" spans="1:6">
+    <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1751,7 +1749,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" ht="20.4" spans="1:6">
+    <row r="4" spans="1:6">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1771,7 +1769,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="20.4" spans="1:6">
+    <row r="5" spans="1:6">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1791,7 +1789,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="20.4" spans="1:6">
+    <row r="6" spans="1:6">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1811,7 +1809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="20.4" spans="1:6">
+    <row r="7" spans="1:6">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1831,7 +1829,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" ht="20.4" spans="1:6">
+    <row r="8" spans="1:6">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1851,7 +1849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="20.4" spans="1:6">
+    <row r="9" spans="1:6">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1871,7 +1869,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" ht="20.4" spans="1:6">
+    <row r="10" spans="1:6">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1891,7 +1889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" ht="20.4" spans="1:6">
+    <row r="11" spans="1:6">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1911,7 +1909,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" ht="20.4" spans="1:6">
+    <row r="12" spans="1:6">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1931,7 +1929,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" ht="20.4" spans="1:6">
+    <row r="13" spans="1:6">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1951,7 +1949,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" ht="20.4" spans="1:6">
+    <row r="14" spans="1:6">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1971,7 +1969,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" ht="20.4" spans="1:6">
+    <row r="15" spans="1:6">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1991,7 +1989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" ht="20.4" spans="1:6">
+    <row r="16" spans="1:6">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2011,7 +2009,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" ht="20.4" spans="1:6">
+    <row r="17" spans="1:6">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2031,7 +2029,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" ht="20.4" spans="1:6">
+    <row r="18" spans="1:6">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2051,7 +2049,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" ht="20.4" spans="1:6">
+    <row r="19" spans="1:6">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2071,7 +2069,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" ht="20.4" spans="1:6">
+    <row r="20" spans="1:6">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2091,7 +2089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" ht="20.4" spans="1:6">
+    <row r="21" spans="1:6">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -2111,7 +2109,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" ht="20.4" spans="1:6">
+    <row r="22" spans="1:6">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -2131,7 +2129,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" ht="20.4" spans="1:6">
+    <row r="23" spans="1:6">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -2151,7 +2149,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" ht="20.4" spans="1:6">
+    <row r="24" spans="1:6">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2171,7 +2169,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" ht="20.4" spans="1:6">
+    <row r="25" spans="1:6">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2191,7 +2189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" ht="20.4" spans="1:6">
+    <row r="26" spans="1:6">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -2211,7 +2209,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" ht="20.4" spans="1:6">
+    <row r="27" spans="1:6">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -2231,7 +2229,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" ht="20.4" spans="1:6">
+    <row r="28" spans="1:6">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -2251,7 +2249,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" ht="20.4" spans="1:6">
+    <row r="29" spans="1:6">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -2271,7 +2269,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" ht="20.4" spans="1:6">
+    <row r="30" spans="1:6">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -2291,7 +2289,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" ht="20.4" spans="1:6">
+    <row r="31" spans="1:6">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -2311,7 +2309,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" ht="20.4" spans="1:6">
+    <row r="32" spans="1:6">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -2331,7 +2329,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" ht="20.4" spans="1:6">
+    <row r="33" spans="1:6">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -2351,7 +2349,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" ht="20.4" spans="1:6">
+    <row r="34" spans="1:6">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -2371,7 +2369,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" ht="20.4" spans="1:6">
+    <row r="35" spans="1:6">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -2391,7 +2389,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" ht="20.4" spans="1:6">
+    <row r="36" spans="1:6">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -2411,7 +2409,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" ht="20.4" spans="1:6">
+    <row r="37" spans="1:6">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -2431,7 +2429,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" ht="20.4" spans="1:6">
+    <row r="38" spans="1:6">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -2451,7 +2449,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" ht="20.4" spans="1:6">
+    <row r="39" spans="1:6">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -2471,7 +2469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" ht="20.4" spans="1:6">
+    <row r="40" spans="1:6">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -2491,7 +2489,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" ht="20.4" spans="1:6">
+    <row r="41" spans="1:6">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -2511,7 +2509,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" ht="20.4" spans="1:6">
+    <row r="42" spans="1:6">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -2531,7 +2529,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" ht="20.4" spans="1:6">
+    <row r="43" spans="1:6">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -2551,7 +2549,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" ht="20.4" spans="1:6">
+    <row r="44" spans="1:6">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2571,7 +2569,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" ht="20.4" spans="1:6">
+    <row r="45" spans="1:6">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2591,7 +2589,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" ht="20.4" spans="1:6">
+    <row r="46" spans="1:6">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -2611,7 +2609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" ht="20.4" spans="1:6">
+    <row r="47" spans="1:6">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2631,7 +2629,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" ht="20.4" spans="1:6">
+    <row r="48" spans="1:6">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2651,7 +2649,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" ht="20.4" spans="1:6">
+    <row r="49" spans="1:6">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2671,7 +2669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" ht="20.4" spans="1:6">
+    <row r="50" spans="1:6">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2691,7 +2689,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" ht="20.4" spans="1:6">
+    <row r="51" spans="1:6">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -2711,7 +2709,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" ht="20.4" spans="1:6">
+    <row r="52" spans="1:6">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -2731,7 +2729,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" ht="20.4" spans="1:6">
+    <row r="53" spans="1:6">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -2751,7 +2749,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" ht="20.4" spans="1:6">
+    <row r="54" spans="1:6">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -2771,7 +2769,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" ht="20.4" spans="1:6">
+    <row r="55" spans="1:6">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -2791,7 +2789,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" ht="20.4" spans="1:6">
+    <row r="56" spans="1:6">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -2811,7 +2809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" ht="20.4" spans="1:6">
+    <row r="57" spans="1:6">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -2831,7 +2829,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" ht="20.4" spans="1:6">
+    <row r="58" spans="1:6">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -2851,7 +2849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" ht="20.4" spans="1:6">
+    <row r="59" spans="1:6">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -2871,7 +2869,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" ht="20.4" spans="1:6">
+    <row r="60" spans="1:6">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -2891,7 +2889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" ht="20.4" spans="1:6">
+    <row r="61" spans="1:6">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -2911,7 +2909,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" ht="20.4" spans="1:6">
+    <row r="62" spans="1:6">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -2931,7 +2929,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" ht="20.4" spans="1:6">
+    <row r="63" spans="1:6">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -2951,7 +2949,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" ht="20.4" spans="1:6">
+    <row r="64" spans="1:6">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -2971,7 +2969,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" ht="20.4" spans="1:6">
+    <row r="65" spans="1:6">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -2991,7 +2989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" ht="20.4" spans="1:6">
+    <row r="66" spans="1:6">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -3011,7 +3009,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" ht="20.4" spans="1:6">
+    <row r="67" spans="1:6">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -3031,7 +3029,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="68" ht="20.4" spans="1:6">
+    <row r="68" spans="1:6">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -3051,7 +3049,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="69" ht="20.4" spans="1:6">
+    <row r="69" spans="1:6">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -3071,7 +3069,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" ht="20.4" spans="1:6">
+    <row r="70" spans="1:6">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -3091,7 +3089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" ht="20.4" spans="1:6">
+    <row r="71" spans="1:6">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -3111,7 +3109,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" ht="20.4" spans="1:6">
+    <row r="72" spans="1:6">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -3131,7 +3129,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="73" ht="20.4" spans="1:6">
+    <row r="73" spans="1:6">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -3151,7 +3149,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" ht="20.4" spans="1:6">
+    <row r="74" spans="1:6">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -3171,7 +3169,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" ht="20.4" spans="1:6">
+    <row r="75" spans="1:6">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -3191,7 +3189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" ht="20.4" spans="1:6">
+    <row r="76" spans="1:6">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -3211,7 +3209,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" ht="20.4" spans="1:6">
+    <row r="77" spans="1:6">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -3231,7 +3229,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" ht="20.4" spans="1:6">
+    <row r="78" spans="1:6">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -3251,7 +3249,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" ht="20.4" spans="1:6">
+    <row r="79" spans="1:6">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -3271,7 +3269,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" ht="20.4" spans="1:6">
+    <row r="80" spans="1:6">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -3291,7 +3289,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" ht="20.4" spans="1:6">
+    <row r="81" spans="1:6">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -3311,7 +3309,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" ht="20.4" spans="1:6">
+    <row r="82" spans="1:6">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -3331,7 +3329,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" ht="20.4" spans="1:6">
+    <row r="83" spans="1:6">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -3351,7 +3349,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" ht="20.4" spans="1:6">
+    <row r="84" spans="1:6">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -3371,7 +3369,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" ht="20.4" spans="1:6">
+    <row r="85" spans="1:6">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -3391,7 +3389,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" ht="20.4" spans="1:6">
+    <row r="86" spans="1:6">
       <c r="A86" s="1">
         <v>85</v>
       </c>
@@ -3411,7 +3409,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" ht="20.4" spans="1:6">
+    <row r="87" spans="1:6">
       <c r="A87" s="1">
         <v>86</v>
       </c>
@@ -3431,7 +3429,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" ht="20.4" spans="1:6">
+    <row r="88" spans="1:6">
       <c r="A88" s="1">
         <v>87</v>
       </c>
@@ -3451,7 +3449,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" ht="20.4" spans="1:6">
+    <row r="89" spans="1:6">
       <c r="A89" s="1">
         <v>88</v>
       </c>
@@ -3471,7 +3469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" ht="20.4" spans="1:6">
+    <row r="90" spans="1:6">
       <c r="A90" s="1">
         <v>89</v>
       </c>
@@ -3491,7 +3489,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="91" ht="20.4" spans="1:6">
+    <row r="91" spans="1:6">
       <c r="A91" s="1">
         <v>90</v>
       </c>
@@ -3511,7 +3509,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" ht="20.4" spans="1:6">
+    <row r="92" spans="1:6">
       <c r="A92" s="1">
         <v>91</v>
       </c>
@@ -3531,7 +3529,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="93" ht="20.4" spans="1:6">
+    <row r="93" spans="1:6">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -3551,7 +3549,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" ht="20.4" spans="1:6">
+    <row r="94" spans="1:6">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -3571,7 +3569,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" ht="20.4" spans="1:6">
+    <row r="95" spans="1:6">
       <c r="A95" s="1">
         <v>94</v>
       </c>
@@ -3591,7 +3589,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" ht="20.4" spans="1:6">
+    <row r="96" spans="1:6">
       <c r="A96" s="1">
         <v>95</v>
       </c>
@@ -3611,7 +3609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" ht="20.4" spans="1:6">
+    <row r="97" spans="1:6">
       <c r="A97" s="1">
         <v>96</v>
       </c>
@@ -3631,7 +3629,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" ht="20.4" spans="1:6">
+    <row r="98" spans="1:6">
       <c r="A98" s="1">
         <v>97</v>
       </c>
@@ -3651,7 +3649,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="99" ht="20.4" spans="1:6">
+    <row r="99" spans="1:6">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -3671,7 +3669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" ht="20.4" spans="1:6">
+    <row r="100" spans="1:6">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -3691,7 +3689,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" ht="20.4" spans="1:6">
+    <row r="101" spans="1:6">
       <c r="A101" s="1">
         <v>100</v>
       </c>
@@ -3711,7 +3709,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="102" ht="20.4" spans="1:6">
+    <row r="102" spans="1:6">
       <c r="A102" s="1">
         <v>101</v>
       </c>
@@ -3731,7 +3729,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="103" ht="20.4" spans="1:6">
+    <row r="103" spans="1:6">
       <c r="A103" s="1">
         <v>102</v>
       </c>
@@ -3739,24 +3737,24 @@
         <v>155</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="104" ht="20.4" spans="1:6">
+    <row r="104" spans="1:6">
       <c r="A104" s="1">
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>44</v>
@@ -3771,247 +3769,247 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" ht="20.4" spans="1:6">
+    <row r="105" spans="1:6">
       <c r="A105" s="1">
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>44</v>
+        <v>145</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>22</v>
+        <v>148</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="106" ht="20.4" spans="1:6">
+    <row r="106" spans="1:6">
       <c r="A106" s="1">
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>89</v>
+        <v>148</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="107" ht="20.4" spans="1:6">
+    <row r="107" spans="1:6">
       <c r="A107" s="1">
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>19</v>
+        <v>146</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="108" ht="20.4" spans="1:6">
+    <row r="108" spans="1:6">
       <c r="A108" s="1">
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>145</v>
+        <v>49</v>
       </c>
       <c r="D108" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>148</v>
+        <v>50</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="109" ht="20.4" spans="1:6">
+    <row r="109" spans="1:6">
       <c r="A109" s="1">
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>145</v>
+        <v>49</v>
       </c>
       <c r="D109" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>148</v>
+        <v>50</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="110" ht="20.4" spans="1:6">
+    <row r="110" spans="1:6">
       <c r="A110" s="1">
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>146</v>
+        <v>58</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="111" ht="20.4" spans="1:6">
+    <row r="111" spans="1:6">
       <c r="A111" s="1">
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>50</v>
+        <v>128</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="112" ht="20.4" spans="1:6">
+    <row r="112" spans="1:6">
       <c r="A112" s="1">
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="113" ht="20.4" spans="1:6">
+    <row r="113" spans="1:6">
       <c r="A113" s="1">
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="D113" s="1" t="s">
         <v>122</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>58</v>
+        <v>167</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="114" ht="20.4" spans="1:6">
+    <row r="114" spans="1:6">
       <c r="A114" s="1">
         <v>113</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>103</v>
+        <v>49</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>128</v>
+        <v>71</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="115" ht="20.4" spans="1:6">
+    <row r="115" spans="1:6">
       <c r="A115" s="1">
         <v>114</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>103</v>
+        <v>49</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="116" ht="20.4" spans="1:6">
+    <row r="116" spans="1:6">
       <c r="A116" s="1">
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>171</v>
+        <v>45</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="117" ht="20.4" spans="1:6">
+    <row r="117" spans="1:6">
       <c r="A117" s="1">
         <v>116</v>
       </c>
@@ -4019,19 +4017,19 @@
         <v>172</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>49</v>
+        <v>171</v>
       </c>
       <c r="D117" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="118" ht="20.4" spans="1:6">
+    <row r="118" spans="1:6">
       <c r="A118" s="1">
         <v>117</v>
       </c>
@@ -4051,7 +4049,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119" ht="20.4" spans="1:6">
+    <row r="119" spans="1:6">
       <c r="A119" s="1">
         <v>118</v>
       </c>
@@ -4059,19 +4057,19 @@
         <v>174</v>
       </c>
       <c r="C119" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E119" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D119" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E119" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="F119" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="120" ht="20.4" spans="1:6">
+    <row r="120" spans="1:6">
       <c r="A120" s="1">
         <v>119</v>
       </c>
@@ -4079,19 +4077,19 @@
         <v>176</v>
       </c>
       <c r="C120" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E120" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="D120" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E120" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="F120" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="121" ht="20.4" spans="1:6">
+    <row r="121" spans="1:6">
       <c r="A121" s="1">
         <v>120</v>
       </c>
@@ -4105,13 +4103,13 @@
         <v>8</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>71</v>
+        <v>175</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="122" ht="20.4" spans="1:6">
+    <row r="122" spans="1:6">
       <c r="A122" s="1">
         <v>121</v>
       </c>
@@ -4125,18 +4123,18 @@
         <v>8</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>179</v>
+        <v>101</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="123" ht="20.4" spans="1:6">
+    <row r="123" spans="1:6">
       <c r="A123" s="1">
         <v>122</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>49</v>
@@ -4145,38 +4143,38 @@
         <v>8</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F123" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="124" ht="20.4" spans="1:6">
+    <row r="124" spans="1:6">
       <c r="A124" s="1">
         <v>123</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>49</v>
+        <v>171</v>
       </c>
       <c r="D124" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>179</v>
+        <v>45</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="125" ht="20.4" spans="1:6">
+    <row r="125" spans="1:6">
       <c r="A125" s="1">
         <v>124</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>49</v>
@@ -4185,18 +4183,18 @@
         <v>8</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="126" ht="20.4" spans="1:6">
+    <row r="126" spans="1:6">
       <c r="A126" s="1">
         <v>125</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>49</v>
@@ -4205,141 +4203,141 @@
         <v>8</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>179</v>
+        <v>71</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="127" ht="20.4" spans="1:6">
+    <row r="127" spans="1:6">
       <c r="A127" s="1">
         <v>126</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>175</v>
+        <v>49</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="128" ht="20.4" spans="1:6">
+    <row r="128" spans="1:6">
       <c r="A128" s="1">
         <v>127</v>
       </c>
       <c r="B128" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C128" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="C128" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="D128" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>50</v>
+        <v>186</v>
       </c>
       <c r="F128" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="129" ht="20.4" spans="1:6">
+    <row r="129" spans="1:6">
       <c r="A129" s="1">
         <v>128</v>
       </c>
       <c r="B129" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E129" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C129" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D129" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E129" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="F129" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="130" ht="20.4" spans="1:6">
+    <row r="130" spans="1:6">
       <c r="A130" s="1">
         <v>129</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="F130" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="131" ht="20.4" spans="1:6">
+    <row r="131" spans="1:6">
       <c r="A131" s="1">
         <v>130</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>189</v>
+        <v>81</v>
       </c>
       <c r="D131" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="F131" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="132" ht="20.4" spans="1:6">
+    <row r="132" spans="1:6">
       <c r="A132" s="1">
         <v>131</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>189</v>
+        <v>81</v>
       </c>
       <c r="D132" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="133" ht="20.4" spans="1:6">
+    <row r="133" spans="1:6">
       <c r="A133" s="1">
         <v>132</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>8</v>
@@ -4351,12 +4349,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" ht="20.4" spans="1:6">
+    <row r="134" spans="1:6">
       <c r="A134" s="1">
         <v>133</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>81</v>
@@ -4365,21 +4363,21 @@
         <v>8</v>
       </c>
       <c r="E134" s="1" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="F134" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="135" ht="20.4" spans="1:6">
+    <row r="135" spans="1:6">
       <c r="A135" s="1">
         <v>134</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="D135" s="1" t="s">
         <v>8</v>
@@ -4391,27 +4389,27 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" ht="20.4" spans="1:6">
+    <row r="136" spans="1:6">
       <c r="A136" s="1">
         <v>135</v>
       </c>
       <c r="B136" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C136" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="C136" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="D136" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E136" s="1" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="F136" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="137" ht="20.4" spans="1:6">
+    <row r="137" spans="1:6">
       <c r="A137" s="1">
         <v>136</v>
       </c>
@@ -4419,19 +4417,19 @@
         <v>196</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>81</v>
+        <v>195</v>
       </c>
       <c r="D137" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="F137" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="138" ht="20.4" spans="1:6">
+    <row r="138" spans="1:6">
       <c r="A138" s="1">
         <v>137</v>
       </c>
@@ -4439,19 +4437,19 @@
         <v>197</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>49</v>
+        <v>195</v>
       </c>
       <c r="D138" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="139" ht="20.4" spans="1:6">
+    <row r="139" spans="1:6">
       <c r="A139" s="1">
         <v>138</v>
       </c>
@@ -4459,7 +4457,7 @@
         <v>198</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D139" s="1" t="s">
         <v>8</v>
@@ -4471,87 +4469,87 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" ht="20.4" spans="1:6">
+    <row r="140" spans="1:6">
       <c r="A140" s="1">
         <v>139</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>199</v>
+        <v>138</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="141" ht="20.4" spans="1:6">
+    <row r="141" spans="1:6">
       <c r="A141" s="1">
         <v>140</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>199</v>
+        <v>61</v>
       </c>
       <c r="D141" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="142" ht="20.4" spans="1:6">
+    <row r="142" spans="1:6">
       <c r="A142" s="1">
         <v>141</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>199</v>
+        <v>61</v>
       </c>
       <c r="D142" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="143" ht="20.4" spans="1:6">
+    <row r="143" spans="1:6">
       <c r="A143" s="1">
         <v>142</v>
       </c>
       <c r="B143" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E143" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C143" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="D143" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E143" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="F143" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="144" ht="20.4" spans="1:6">
+    <row r="144" spans="1:6">
       <c r="A144" s="1">
         <v>143</v>
       </c>
@@ -4565,13 +4563,13 @@
         <v>8</v>
       </c>
       <c r="E144" s="1" t="s">
-        <v>15</v>
+        <v>203</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="145" ht="20.4" spans="1:6">
+    <row r="145" spans="1:6">
       <c r="A145" s="1">
         <v>144</v>
       </c>
@@ -4579,39 +4577,39 @@
         <v>205</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>45</v>
+        <v>206</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="146" ht="20.4" spans="1:6">
+    <row r="146" spans="1:6">
       <c r="A146" s="1">
         <v>145</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>207</v>
+        <v>58</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="147" ht="20.4" spans="1:6">
+    <row r="147" spans="1:6">
       <c r="A147" s="1">
         <v>146</v>
       </c>
@@ -4619,19 +4617,19 @@
         <v>208</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D147" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>207</v>
+        <v>58</v>
       </c>
       <c r="F147" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="148" ht="20.4" spans="1:6">
+    <row r="148" spans="1:6">
       <c r="A148" s="1">
         <v>147</v>
       </c>
@@ -4639,139 +4637,139 @@
         <v>209</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>103</v>
+        <v>195</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>210</v>
+        <v>12</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="149" ht="20.4" spans="1:6">
+    <row r="149" spans="1:6">
       <c r="A149" s="1">
         <v>148</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>57</v>
+        <v>195</v>
       </c>
       <c r="D149" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="150" ht="20.4" spans="1:6">
+    <row r="150" spans="1:6">
       <c r="A150" s="1">
         <v>149</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>57</v>
+        <v>195</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="F150" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="151" ht="20.4" spans="1:6">
+    <row r="151" spans="1:6">
       <c r="A151" s="1">
         <v>150</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D151" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="152" ht="20.4" spans="1:6">
+    <row r="152" spans="1:6">
       <c r="A152" s="1">
         <v>151</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>199</v>
+        <v>171</v>
       </c>
       <c r="D152" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="F152" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="153" ht="20.4" spans="1:6">
+    <row r="153" spans="1:6">
       <c r="A153" s="1">
         <v>152</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>199</v>
+        <v>103</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>15</v>
+        <v>130</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="154" ht="20.4" spans="1:6">
+    <row r="154" spans="1:6">
       <c r="A154" s="1">
         <v>153</v>
       </c>
       <c r="B154" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E154" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="C154" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="D154" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E154" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="F154" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="155" ht="20.4" spans="1:6">
+    <row r="155" spans="1:6">
       <c r="A155" s="1">
         <v>154</v>
       </c>
@@ -4779,19 +4777,19 @@
         <v>217</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>175</v>
+        <v>34</v>
       </c>
       <c r="D155" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="F155" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="156" ht="20.4" spans="1:6">
+    <row r="156" spans="1:6">
       <c r="A156" s="1">
         <v>155</v>
       </c>
@@ -4799,19 +4797,19 @@
         <v>218</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>103</v>
+        <v>34</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>130</v>
+        <v>66</v>
       </c>
       <c r="F156" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="157" ht="20.4" spans="1:6">
+    <row r="157" spans="1:6">
       <c r="A157" s="1">
         <v>156</v>
       </c>
@@ -4819,84 +4817,84 @@
         <v>219</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>103</v>
+        <v>34</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>220</v>
+        <v>66</v>
       </c>
       <c r="F157" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="158" ht="20.4" spans="1:6">
+    <row r="158" spans="1:6">
       <c r="A158" s="1">
         <v>157</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="D158" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>89</v>
+        <v>175</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="159" ht="20.4" spans="1:6">
+    <row r="159" spans="1:6">
       <c r="A159" s="1">
         <v>158</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="D159" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>66</v>
+        <v>175</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="160" ht="20.4" spans="1:6">
+    <row r="160" spans="1:6">
       <c r="A160" s="1">
         <v>159</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="D160" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="F160" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="161" ht="20.4" spans="1:6">
+    <row r="161" spans="1:6">
       <c r="A161" s="1">
         <v>160</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>103</v>
@@ -4905,18 +4903,18 @@
         <v>8</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F161" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="162" ht="20.4" spans="1:6">
+    <row r="162" spans="1:6">
       <c r="A162" s="1">
         <v>161</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>103</v>
@@ -4925,167 +4923,167 @@
         <v>8</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>179</v>
+        <v>50</v>
       </c>
       <c r="F162" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="163" ht="20.4" spans="1:6">
+    <row r="163" spans="1:6">
       <c r="A163" s="1">
         <v>162</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>50</v>
+        <v>128</v>
       </c>
       <c r="F163" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="164" ht="20.4" spans="1:6">
+    <row r="164" spans="1:6">
       <c r="A164" s="1">
         <v>163</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>179</v>
+        <v>58</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="165" ht="20.4" spans="1:6">
+    <row r="165" spans="1:6">
       <c r="A165" s="1">
         <v>164</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>50</v>
+        <v>216</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="166" ht="20.4" spans="1:6">
+    <row r="166" spans="1:6">
       <c r="A166" s="1">
         <v>165</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>103</v>
+        <v>138</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E166" s="1" t="s">
-        <v>128</v>
+        <v>22</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="167" ht="20.4" spans="1:6">
+    <row r="167" spans="1:6">
       <c r="A167" s="1">
         <v>166</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>103</v>
+        <v>138</v>
       </c>
       <c r="D167" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E167" s="1" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="F167" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="168" ht="20.4" spans="1:6">
+    <row r="168" spans="1:6">
       <c r="A168" s="1">
         <v>167</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D168" s="1" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>220</v>
+        <v>50</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="169" ht="20.4" spans="1:6">
+    <row r="169" spans="1:6">
       <c r="A169" s="1">
         <v>168</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="D169" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="F169" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="170" ht="20.4" spans="1:6">
+    <row r="170" spans="1:6">
       <c r="A170" s="1">
         <v>169</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="D170" s="1" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>22</v>
+        <v>206</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>10</v>

</xml_diff>